<commit_message>
M 12600512.xlsx  M notebooks/CAP776_12600512.ipynb  M notebooks/python_module.ipynb
</commit_message>
<xml_diff>
--- a/12600512.xlsx
+++ b/12600512.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\vaults\my vault\01-academics\01-semester\02-cap776-python\04-assignments\daily-activity-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0F38389-EFA7-4773-9D39-8C26DD93EB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9262BE2-18B6-485D-9D8C-C74CB8C2A713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -239,6 +239,15 @@
   </si>
   <si>
     <t>I start solving problems in codewars</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>I did well in my DBMS CA</t>
+  </si>
+  <si>
+    <t>I registered for my first hackathon</t>
   </si>
 </sst>
 </file>
@@ -1854,92 +1863,184 @@
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="10" t="str">
+      <c r="A25" s="8">
+        <v>46270</v>
+      </c>
+      <c r="B25" s="9">
+        <v>460</v>
+      </c>
+      <c r="C25" s="9">
+        <v>0</v>
+      </c>
+      <c r="D25" s="9">
+        <v>200</v>
+      </c>
+      <c r="E25" s="9">
+        <v>150</v>
+      </c>
+      <c r="F25" s="9">
+        <v>0</v>
+      </c>
+      <c r="G25" s="9">
+        <v>0</v>
+      </c>
+      <c r="H25" s="9">
+        <v>0</v>
+      </c>
+      <c r="I25" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="10" t="str">
+        <v>810</v>
+      </c>
+      <c r="J25" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
+        <v>630</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M25" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N25" s="12"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="8"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="10" t="str">
+      <c r="A26" s="8">
+        <v>46271</v>
+      </c>
+      <c r="B26" s="9">
+        <v>460</v>
+      </c>
+      <c r="C26" s="9">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9">
+        <v>240</v>
+      </c>
+      <c r="E26" s="9">
+        <v>120</v>
+      </c>
+      <c r="F26" s="9">
+        <v>0</v>
+      </c>
+      <c r="G26" s="9">
+        <v>0</v>
+      </c>
+      <c r="H26" s="9">
+        <v>0</v>
+      </c>
+      <c r="I26" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="10" t="str">
+        <v>820</v>
+      </c>
+      <c r="J26" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
+        <v>620</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M26" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N26" s="12"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="8"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="10" t="str">
+      <c r="A27" s="8">
+        <v>46272</v>
+      </c>
+      <c r="B27" s="9">
+        <v>420</v>
+      </c>
+      <c r="C27" s="9">
+        <v>0</v>
+      </c>
+      <c r="D27" s="9">
+        <v>300</v>
+      </c>
+      <c r="E27" s="9">
+        <v>200</v>
+      </c>
+      <c r="F27" s="9">
+        <v>200</v>
+      </c>
+      <c r="G27" s="9">
+        <v>4</v>
+      </c>
+      <c r="H27" s="9">
+        <v>0</v>
+      </c>
+      <c r="I27" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="10" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J27" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="12"/>
+        <v>320</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L27" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M27" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="N27" s="12" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="10" t="str">
+      <c r="A28" s="8">
+        <v>46273</v>
+      </c>
+      <c r="B28" s="9">
+        <v>420</v>
+      </c>
+      <c r="C28" s="9">
+        <v>0</v>
+      </c>
+      <c r="D28" s="9">
+        <v>240</v>
+      </c>
+      <c r="E28" s="9">
+        <v>60</v>
+      </c>
+      <c r="F28" s="9">
+        <v>350</v>
+      </c>
+      <c r="G28" s="9">
+        <v>7</v>
+      </c>
+      <c r="H28" s="9">
+        <v>0</v>
+      </c>
+      <c r="I28" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="10" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J28" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="12"/>
+        <v>370</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="M28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N28" s="12" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>

</xml_diff>

<commit_message>
M 12600512.xlsx  M minor_project_01_py.ipynb
</commit_message>
<xml_diff>
--- a/12600512.xlsx
+++ b/12600512.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\vaults\my vault\01-academics\01-semester\02-cap776-python\04-assignments\daily-activity-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39CC583-1AFF-4EA9-A2EF-84214A5DC7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B86E612-CFC8-409A-AAC6-A1D54270E7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2519,69 +2519,135 @@
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="8"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="10" t="str">
+      <c r="A39" s="8">
+        <v>46284</v>
+      </c>
+      <c r="B39" s="9">
+        <v>420</v>
+      </c>
+      <c r="C39" s="9">
+        <v>0</v>
+      </c>
+      <c r="D39" s="9">
+        <v>180</v>
+      </c>
+      <c r="E39" s="9">
+        <v>60</v>
+      </c>
+      <c r="F39" s="9">
+        <v>0</v>
+      </c>
+      <c r="G39" s="9">
+        <v>0</v>
+      </c>
+      <c r="H39" s="9">
+        <v>0</v>
+      </c>
+      <c r="I39" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="10" t="str">
+        <v>660</v>
+      </c>
+      <c r="J39" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
-      <c r="M39" s="11"/>
+        <v>780</v>
+      </c>
+      <c r="K39" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L39" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M39" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N39" s="12"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="8"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="10" t="str">
+      <c r="A40" s="8">
+        <v>46285</v>
+      </c>
+      <c r="B40" s="9">
+        <v>400</v>
+      </c>
+      <c r="C40" s="9">
+        <v>0</v>
+      </c>
+      <c r="D40" s="9">
+        <v>200</v>
+      </c>
+      <c r="E40" s="9">
+        <v>150</v>
+      </c>
+      <c r="F40" s="9">
+        <v>0</v>
+      </c>
+      <c r="G40" s="9">
+        <v>0</v>
+      </c>
+      <c r="H40" s="9">
+        <v>0</v>
+      </c>
+      <c r="I40" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="10" t="str">
+        <v>750</v>
+      </c>
+      <c r="J40" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="11"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="11"/>
+        <v>690</v>
+      </c>
+      <c r="K40" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L40" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M40" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N40" s="12"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="8"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="10" t="str">
+      <c r="A41" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B41" s="9">
+        <v>390</v>
+      </c>
+      <c r="C41" s="9">
+        <v>0</v>
+      </c>
+      <c r="D41" s="9">
+        <v>260</v>
+      </c>
+      <c r="E41" s="9">
+        <v>120</v>
+      </c>
+      <c r="F41" s="9">
+        <v>200</v>
+      </c>
+      <c r="G41" s="9">
+        <v>4</v>
+      </c>
+      <c r="H41" s="9">
+        <v>0</v>
+      </c>
+      <c r="I41" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="10" t="str">
+        <v>970</v>
+      </c>
+      <c r="J41" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="11"/>
-      <c r="L41" s="11"/>
-      <c r="M41" s="11"/>
+        <v>470</v>
+      </c>
+      <c r="K41" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L41" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M41" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N41" s="12"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>